<commit_message>
Record the Home and Profile checks that do not clear the phone.
About, Licences and Privacy open on the device, and the language and city changes were put back. Delete my data was not pressed.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tests/M5-home-profile.xlsx
+++ b/tests/M5-home-profile.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="2" max="2"/>
@@ -454,6 +454,7 @@
     <col width="24.140625" customWidth="1" min="7" max="7"/>
     <col width="26.5703125" customWidth="1" min="8" max="8"/>
     <col width="30.42578125" customWidth="1" min="9" max="9"/>
+    <col width="62" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -512,6 +513,11 @@
           <t>Test Type</t>
         </is>
       </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Result</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="57.95" customHeight="1">
       <c r="A2" s="3" t="n">
@@ -556,6 +562,11 @@
       </c>
       <c r="J2" s="4" t="inlineStr"/>
       <c r="K2" s="4" t="inlineStr"/>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. Good afternoon, then Mon 14 Sep · śukla tṛtīyā · Hyderabad. No clock.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="57.95" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -600,6 +611,11 @@
       </c>
       <c r="J3" s="4" t="inlineStr"/>
       <c r="K3" s="4" t="inlineStr"/>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS on the day. Home shows Vinayaka Chavithi and Start the puja. The day before the festival was not opened.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="57.95" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -645,6 +661,11 @@
       </c>
       <c r="J4" s="4" t="inlineStr"/>
       <c r="K4" s="4" t="inlineStr"/>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. The bar reads Ganapati mula mantra and 4 more.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="57.95" customHeight="1">
       <c r="A5" s="3" t="n">
@@ -689,6 +710,11 @@
       </c>
       <c r="J5" s="4" t="inlineStr"/>
       <c r="K5" s="4" t="inlineStr"/>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run. The phone already has japams.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="57.95" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -734,6 +760,11 @@
       </c>
       <c r="J6" s="4" t="inlineStr"/>
       <c r="K6" s="4" t="inlineStr"/>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS for Telugu. Switching the app language updated Home, Stories, the god page and an open story. It was set back to English. Hindi was not walked across every module this pass.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="57.95" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -779,6 +810,11 @@
       </c>
       <c r="J7" s="4" t="inlineStr"/>
       <c r="K7" s="4" t="inlineStr"/>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. Maharashtra and Mumbai saved, and the home line followed. Restored to Telangana and Hyderabad.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="57.95" customHeight="1">
       <c r="A8" s="3" t="n">
@@ -824,6 +860,11 @@
       </c>
       <c r="J8" s="4" t="inlineStr"/>
       <c r="K8" s="4" t="inlineStr"/>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run. Delete my data was not pressed.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="57.95" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -869,6 +910,11 @@
       </c>
       <c r="J9" s="4" t="inlineStr"/>
       <c r="K9" s="4" t="inlineStr"/>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PASS. About shows app version 0.3.0-dev and content pack 20261024.1303. Licences lists the four fonts and the libraries. Privacy opens offline and says the body is the English draft.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="57.95" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -914,6 +960,11 @@
       </c>
       <c r="J10" s="4" t="inlineStr"/>
       <c r="K10" s="4" t="inlineStr"/>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Home at 200% shows the greeting, the date line, the festival card and the sādhana bar. The god grid, the god page and the katha card were checked earlier. Not every route was screenshotted.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="57.95" customHeight="1">
       <c r="A11" s="3" t="n">
@@ -959,6 +1010,11 @@
       </c>
       <c r="J11" s="4" t="inlineStr"/>
       <c r="K11" s="4" t="inlineStr"/>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Back and Home are words. The god card reads Ganesha, 4 stories and the katha card reads Chavithi katha, 2 parts. A full Home to Puja TalkBack walk was not done.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="57.95" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -1002,6 +1058,11 @@
       </c>
       <c r="J12" s="4" t="inlineStr"/>
       <c r="K12" s="4" t="inlineStr"/>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not run. A 30-minute monkey can press Delete my data.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="57.95" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -1045,6 +1106,11 @@
       </c>
       <c r="J13" s="4" t="inlineStr"/>
       <c r="K13" s="4" t="inlineStr"/>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The manifest has no internet permission. The offering Search button is the one control that opens the browser, and only while online. A network inspector was not attached.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>